<commit_message>
docs: record code hosting as provided (A7)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxscWn9fSBZzY3BEJFGfy4
</commit_message>
<xml_diff>
--- a/docs/sachin-to-provide.xlsx
+++ b/docs/sachin-to-provide.xlsx
@@ -1009,11 +1009,17 @@
       </c>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="13" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>github.com/sachinkuber/marketing.sarathi.gvcc.in (private). Pushed over HTTPS; the SSH key on this machine signs in as gvcc-sharyo, which has no access to it.</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>46299</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -3719,7 +3725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4305,6 +4311,23 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Code hosting (A7)</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Private GitHub repository sachinkuber/marketing.sarathi.gvcc.in</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: Phase 1 spec v5 - per-process brand limit
Approved by the owner on 2026-10-04 after the queue trial showed the
library's global group limit is exceeded under concurrent fetches.
Sections 3, 9.2, 9.3 and 19 only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxscWn9fSBZzY3BEJFGfy4
</commit_message>
<xml_diff>
--- a/docs/sachin-to-provide.xlsx
+++ b/docs/sachin-to-provide.xlsx
@@ -3725,7 +3725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Approved</t>
+          <t>Approved, then replaced by version 5</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
@@ -4229,12 +4229,12 @@
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>Cost currency</t>
+          <t>Phase 1 spec version 5</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Every cost recorded in both US dollars and Indian rupees</t>
+          <t>Approved: per-process brand limit, after the queue trial</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
@@ -4246,12 +4246,12 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Retention of job inputs and notifications</t>
+          <t>Cost currency</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>90 days</t>
+          <t>Every cost recorded in both US dollars and Indian rupees</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -4263,12 +4263,12 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Database schema version 2</t>
+          <t>Retention of job inputs and notifications</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Approved. Later-phase tables stay provisional.</t>
+          <t>90 days</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -4280,12 +4280,12 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>Phased implementation plan version 1</t>
+          <t>Database schema version 2</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Approved, with its assumption that Claude Code builds and the owner reviews</t>
+          <t>Approved. Later-phase tables stay provisional.</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
@@ -4297,12 +4297,12 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Permission to commit (A8)</t>
+          <t>Phased implementation plan version 1</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Approved, with its assumption that Claude Code builds and the owner reviews</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
@@ -4314,15 +4314,32 @@
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
+          <t>Permission to commit (A8)</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
           <t>Code hosting (A7)</t>
         </is>
       </c>
-      <c r="B35" s="11" t="inlineStr">
+      <c r="B36" s="11" t="inlineStr">
         <is>
           <t>Private GitHub repository sachinkuber/marketing.sarathi.gvcc.in</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C36" s="11" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>

</xml_diff>

<commit_message>
docs: Tech stack v2 - ESLint 10.10.0 replaces unsupported 9.39.5
Approved by the owner on 2026-10-04. Phase 1 spec section 3 copies the
new version.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxscWn9fSBZzY3BEJFGfy4
</commit_message>
<xml_diff>
--- a/docs/sachin-to-provide.xlsx
+++ b/docs/sachin-to-provide.xlsx
@@ -3725,7 +3725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4246,12 +4246,12 @@
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Cost currency</t>
+          <t>Tech stack version 2</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Every cost recorded in both US dollars and Indian rupees</t>
+          <t>Approved: ESLint 10.10.0 in place of the unsupported 9.39.5</t>
         </is>
       </c>
       <c r="C31" s="11" t="inlineStr">
@@ -4263,12 +4263,12 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Retention of job inputs and notifications</t>
+          <t>Cost currency</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>90 days</t>
+          <t>Every cost recorded in both US dollars and Indian rupees</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
@@ -4280,12 +4280,12 @@
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>Database schema version 2</t>
+          <t>Retention of job inputs and notifications</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Approved. Later-phase tables stay provisional.</t>
+          <t>90 days</t>
         </is>
       </c>
       <c r="C33" s="11" t="inlineStr">
@@ -4297,12 +4297,12 @@
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Phased implementation plan version 1</t>
+          <t>Database schema version 2</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>Approved, with its assumption that Claude Code builds and the owner reviews</t>
+          <t>Approved. Later-phase tables stay provisional.</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
@@ -4314,12 +4314,12 @@
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Permission to commit (A8)</t>
+          <t>Phased implementation plan version 1</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Approved, with its assumption that Claude Code builds and the owner reviews</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
@@ -4331,15 +4331,32 @@
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
         <is>
+          <t>Permission to commit (A8)</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
           <t>Code hosting (A7)</t>
         </is>
       </c>
-      <c r="B36" s="11" t="inlineStr">
+      <c r="B37" s="11" t="inlineStr">
         <is>
           <t>Private GitHub repository sachinkuber/marketing.sarathi.gvcc.in</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C37" s="11" t="inlineStr">
         <is>
           <t>2026-10-04</t>
         </is>

</xml_diff>

<commit_message>
docs: to-provide list brought up to date (H17 done)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxscWn9fSBZzY3BEJFGfy4
</commit_message>
<xml_diff>
--- a/docs/sachin-to-provide.xlsx
+++ b/docs/sachin-to-provide.xlsx
@@ -3571,11 +3571,17 @@
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G83" s="12" t="n"/>
-      <c r="H83" s="13" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G83" s="12" t="inlineStr">
+        <is>
+          <t>Approved with the Tech stack and Architecture: claude-opus-5-5 for every agent to start.</t>
+        </is>
+      </c>
+      <c r="H83" s="13" t="n">
+        <v>46299</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H83"/>

</xml_diff>